<commit_message>
Updating forensic file tracking doc
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d87909e21b199fc/Documents/BHB-Capstone/Forensic File Tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{DC198764-2EF7-4C00-B63F-195CD3C55462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5404E8CF-B4D2-4478-B2FA-ACA19AE1AD25}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{DC198764-2EF7-4C00-B63F-195CD3C55462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE2914E8-1A2A-471E-98E3-62303EB01474}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
@@ -77,10 +77,10 @@
     <t>No</t>
   </si>
   <si>
-    <t>SIX.dd</t>
-  </si>
-  <si>
     <t>Olivia Hey</t>
+  </si>
+  <si>
+    <t>THREE.dd</t>
   </si>
 </sst>
 </file>
@@ -124,10 +124,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -143,6 +142,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -546,11 +549,11 @@
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="C7" s="2" t="s">
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
         <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
       </c>
       <c r="E7" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Weekly log research log and updated forensic file tracking document week 1o
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d87909e21b199fc/Documents/BHB-Capstone/Forensic File Tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{DC198764-2EF7-4C00-B63F-195CD3C55462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE2914E8-1A2A-471E-98E3-62303EB01474}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="8_{DC198764-2EF7-4C00-B63F-195CD3C55462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97CDA120-660D-458C-A700-DB53FD93EB32}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="17">
   <si>
     <t>File</t>
   </si>
@@ -81,13 +81,22 @@
   </si>
   <si>
     <t>THREE.dd</t>
+  </si>
+  <si>
+    <t>NINE.dd</t>
+  </si>
+  <si>
+    <t>Sam Davies</t>
+  </si>
+  <si>
+    <t>Date Completed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,16 +112,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -120,15 +150,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
+    <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -465,157 +510,197 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58C512E3-CCD5-4663-8B80-5D68DC0D3979}">
-  <dimension ref="B2:M26"/>
+  <dimension ref="B2:Q26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.90625" customWidth="1"/>
-    <col min="3" max="3" width="22.453125" customWidth="1"/>
-    <col min="4" max="4" width="17.7265625" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="22.90625" customWidth="1"/>
-    <col min="7" max="7" width="17.08984375" customWidth="1"/>
-    <col min="8" max="8" width="19.90625" customWidth="1"/>
-    <col min="9" max="9" width="22.6328125" customWidth="1"/>
-    <col min="10" max="10" width="22.54296875" customWidth="1"/>
-    <col min="11" max="11" width="17.81640625" customWidth="1"/>
-    <col min="12" max="12" width="17.6328125" customWidth="1"/>
-    <col min="13" max="13" width="18.36328125" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="15.90625" customWidth="1"/>
+    <col min="4" max="4" width="22.453125" customWidth="1"/>
+    <col min="5" max="5" width="17.7265625" customWidth="1"/>
+    <col min="6" max="6" width="21.7265625" customWidth="1"/>
+    <col min="7" max="7" width="22.6328125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="22.90625" customWidth="1"/>
+    <col min="9" max="9" width="17.08984375" customWidth="1"/>
+    <col min="10" max="10" width="19.90625" customWidth="1"/>
+    <col min="11" max="11" width="22.6328125" customWidth="1"/>
+    <col min="12" max="12" width="22.54296875" style="2" customWidth="1"/>
+    <col min="13" max="13" width="22.54296875" customWidth="1"/>
+    <col min="14" max="14" width="17.81640625" customWidth="1"/>
+    <col min="15" max="15" width="17.6328125" customWidth="1"/>
+    <col min="16" max="16" width="18.36328125" customWidth="1"/>
+    <col min="17" max="17" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B2" s="1"/>
+    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="K2" s="1"/>
-    </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B3" s="1" t="s">
+      <c r="F2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+    </row>
+    <row r="3" spans="2:16" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:16" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="G4" s="1" t="s">
+      <c r="F4" s="1"/>
+      <c r="H4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="I4" s="1"/>
+      <c r="M4" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="N4" s="1"/>
+    </row>
+    <row r="5" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="M5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="P5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="C6" t="s">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="D6" t="s">
         <v>2</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>3</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="C7" t="s">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="D7" t="s">
         <v>13</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="C12" s="1"/>
-    </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="C13" s="1"/>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-    </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B24" s="1" t="s">
+      <c r="F13" s="1"/>
+    </row>
+    <row r="24" spans="2:16" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B24" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="1"/>
-    </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="2:16" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="C25" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
-      <c r="G25" s="1" t="s">
+      <c r="F25" s="1"/>
+      <c r="H25" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K25" s="1" t="s">
+      <c r="I25" s="1"/>
+      <c r="M25" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="N25" s="1"/>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="E26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="H26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="K26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="M26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N26" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="L26" s="1" t="s">
+      <c r="O26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M26" s="1" t="s">
+      <c r="P26" s="1" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated logs, added folders for AI reports, updated forensic file tracking excel
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d87909e21b199fc/Documents/BHB-Capstone/Forensic File Tracking/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Forensic File Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="8_{DC198764-2EF7-4C00-B63F-195CD3C55462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97CDA120-660D-458C-A700-DB53FD93EB32}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0A4A80-8F1B-4F61-9124-47594094783A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
+    <workbookView xWindow="345" yWindow="1215" windowWidth="37770" windowHeight="17970" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="19">
   <si>
     <t>File</t>
   </si>
@@ -90,6 +90,12 @@
   </si>
   <si>
     <t>Date Completed</t>
+  </si>
+  <si>
+    <t>Evidence1.pcap</t>
+  </si>
+  <si>
+    <t>nmap_example.xml</t>
   </si>
 </sst>
 </file>
@@ -187,10 +193,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -510,28 +512,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58C512E3-CCD5-4663-8B80-5D68DC0D3979}">
-  <dimension ref="B2:Q26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:Q29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="15.90625" customWidth="1"/>
-    <col min="4" max="4" width="22.453125" customWidth="1"/>
-    <col min="5" max="5" width="17.7265625" customWidth="1"/>
-    <col min="6" max="6" width="21.7265625" customWidth="1"/>
-    <col min="7" max="7" width="22.6328125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="22.90625" customWidth="1"/>
-    <col min="9" max="9" width="17.08984375" customWidth="1"/>
-    <col min="10" max="10" width="19.90625" customWidth="1"/>
-    <col min="11" max="11" width="22.6328125" customWidth="1"/>
-    <col min="12" max="12" width="22.54296875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="22.54296875" customWidth="1"/>
-    <col min="14" max="14" width="17.81640625" customWidth="1"/>
-    <col min="15" max="15" width="17.6328125" customWidth="1"/>
-    <col min="16" max="16" width="18.36328125" customWidth="1"/>
-    <col min="17" max="17" width="8.7265625" style="2"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="22.85546875" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" customWidth="1"/>
+    <col min="10" max="10" width="19.85546875" customWidth="1"/>
+    <col min="11" max="11" width="22.5703125" customWidth="1"/>
+    <col min="12" max="12" width="22.5703125" style="2" customWidth="1"/>
+    <col min="13" max="13" width="22.5703125" customWidth="1"/>
+    <col min="14" max="14" width="17.85546875" customWidth="1"/>
+    <col min="15" max="15" width="17.5703125" customWidth="1"/>
+    <col min="16" max="16" width="18.42578125" customWidth="1"/>
+    <col min="17" max="17" width="8.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -540,12 +542,12 @@
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
     </row>
-    <row r="3" spans="2:16" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:16" s="2" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:16" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
@@ -561,7 +563,7 @@
       </c>
       <c r="N4" s="1"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C5" s="1" t="s">
         <v>16</v>
       </c>
@@ -599,7 +601,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>2</v>
       </c>
@@ -609,8 +611,11 @@
       <c r="F6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="I6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>13</v>
       </c>
@@ -621,7 +626,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
         <v>14</v>
       </c>
@@ -632,20 +637,20 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="24" spans="2:16" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="2:16" s="2" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:16" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C25" s="1" t="s">
         <v>5</v>
       </c>
@@ -661,7 +666,7 @@
       </c>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C26" s="1" t="s">
         <v>16</v>
       </c>
@@ -697,6 +702,27 @@
       </c>
       <c r="P26" s="1" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="D27" t="s">
+        <v>2</v>
+      </c>
+      <c r="I27" t="s">
+        <v>17</v>
+      </c>
+      <c r="N27" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="D29" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added AI foremost reports, updated forensic file tracking
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Forensic File Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0A4A80-8F1B-4F61-9124-47594094783A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B114DA9-4B84-4D0A-8D1B-FE5CBA1407AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="1215" windowWidth="37770" windowHeight="17970" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21150" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="23">
   <si>
     <t>File</t>
   </si>
@@ -80,9 +80,6 @@
     <t>Olivia Hey</t>
   </si>
   <si>
-    <t>THREE.dd</t>
-  </si>
-  <si>
     <t>NINE.dd</t>
   </si>
   <si>
@@ -96,6 +93,22 @@
   </si>
   <si>
     <t>nmap_example.xml</t>
+  </si>
+  <si>
+    <t>Three.dd</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>gemma4-df:latest</t>
+  </si>
+  <si>
+    <t>AI Model</t>
+  </si>
+  <si>
+    <t>FOREMOST
+w/NinemostV1.py</t>
   </si>
 </sst>
 </file>
@@ -171,11 +184,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -516,7 +533,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
     <col min="4" max="4" width="22.42578125" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" customWidth="1"/>
     <col min="6" max="6" width="21.7109375" customWidth="1"/>
@@ -565,7 +582,7 @@
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>0</v>
@@ -577,7 +594,7 @@
         <v>4</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>0</v>
@@ -589,7 +606,7 @@
         <v>4</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>0</v>
@@ -612,12 +629,12 @@
         <v>11</v>
       </c>
       <c r="I6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
@@ -628,10 +645,10 @@
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
         <v>14</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
       </c>
       <c r="F8" t="s">
         <v>11</v>
@@ -650,9 +667,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="1" t="s">
-        <v>5</v>
+    <row r="25" spans="2:16" ht="45.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="4" t="s">
+        <v>22</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -668,19 +685,19 @@
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C26" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>0</v>
@@ -692,7 +709,7 @@
         <v>4</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N26" s="1" t="s">
         <v>0</v>
@@ -705,24 +722,51 @@
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="C27" s="5">
+        <v>46288</v>
+      </c>
       <c r="D27" t="s">
         <v>2</v>
       </c>
+      <c r="E27" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" t="s">
+        <v>19</v>
+      </c>
       <c r="I27" t="s">
+        <v>16</v>
+      </c>
+      <c r="N27" t="s">
         <v>17</v>
       </c>
-      <c r="N27" t="s">
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="C28" s="5">
+        <v>46288</v>
+      </c>
+      <c r="D28" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="D28" t="s">
+      <c r="E28" t="s">
+        <v>20</v>
+      </c>
+      <c r="F28" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="C29" s="5">
+        <v>46288</v>
+      </c>
+      <c r="D29" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="D29" t="s">
-        <v>14</v>
+      <c r="E29" t="s">
+        <v>20</v>
+      </c>
+      <c r="F29" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated logs, added ALL AI reports, updated file tracking document
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/Forensic File Tracking/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Forensic File Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{1B114DA9-4B84-4D0A-8D1B-FE5CBA1407AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A2667BE-EC4F-4269-B4A3-D11BF509613C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A1BDDFE-A367-400D-A7C2-186AA66F5413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1005" windowWidth="21600" windowHeight="11385" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
+    <workbookView xWindow="38280" yWindow="2910" windowWidth="29040" windowHeight="15990" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="28">
   <si>
     <t>File</t>
   </si>
@@ -87,9 +87,6 @@
   </si>
   <si>
     <t>Date Completed</t>
-  </si>
-  <si>
-    <t>Evidence1.pcap</t>
   </si>
   <si>
     <t>nmap_example.xml</t>
@@ -115,6 +112,18 @@
   </si>
   <si>
     <t>Dave</t>
+  </si>
+  <si>
+    <t>evidence01.pcap</t>
+  </si>
+  <si>
+    <t>evidence02.pcapng</t>
+  </si>
+  <si>
+    <t>SOITnetworkscan.xml</t>
+  </si>
+  <si>
+    <t>28sepServiceScan.xml</t>
   </si>
 </sst>
 </file>
@@ -535,7 +544,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58C512E3-CCD5-4663-8B80-5D68DC0D3979}">
-  <dimension ref="B2:Q29"/>
+  <dimension ref="B2:Q33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -550,7 +559,7 @@
     <col min="11" max="11" width="22.5703125" customWidth="1"/>
     <col min="12" max="12" width="22.5703125" style="2" customWidth="1"/>
     <col min="13" max="13" width="22.5703125" customWidth="1"/>
-    <col min="14" max="14" width="17.85546875" customWidth="1"/>
+    <col min="14" max="14" width="21.140625" customWidth="1"/>
     <col min="15" max="15" width="17.5703125" customWidth="1"/>
     <col min="16" max="16" width="18.42578125" customWidth="1"/>
     <col min="17" max="17" width="8.7109375" style="2"/>
@@ -635,12 +644,12 @@
         <v>11</v>
       </c>
       <c r="I6" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
@@ -652,13 +661,13 @@
         <v>46296</v>
       </c>
       <c r="I7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" t="s">
         <v>23</v>
       </c>
-      <c r="J7" t="s">
-        <v>24</v>
-      </c>
       <c r="K7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.25">
@@ -687,7 +696,7 @@
     </row>
     <row r="25" spans="2:16" ht="45.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C25" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -709,7 +718,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>4</v>
@@ -747,16 +756,34 @@
         <v>2</v>
       </c>
       <c r="E27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F27" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="H27" s="5">
+        <v>46297</v>
       </c>
       <c r="I27" t="s">
+        <v>24</v>
+      </c>
+      <c r="J27" t="s">
+        <v>19</v>
+      </c>
+      <c r="K27" t="s">
+        <v>18</v>
+      </c>
+      <c r="M27" s="5">
+        <v>46297</v>
+      </c>
+      <c r="N27" t="s">
         <v>16</v>
       </c>
-      <c r="N27" t="s">
-        <v>17</v>
+      <c r="O27" t="s">
+        <v>19</v>
+      </c>
+      <c r="P27" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
@@ -764,13 +791,37 @@
         <v>46288</v>
       </c>
       <c r="D28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F28" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="H28" s="5">
+        <v>46297</v>
+      </c>
+      <c r="I28" t="s">
+        <v>25</v>
+      </c>
+      <c r="J28" t="s">
+        <v>19</v>
+      </c>
+      <c r="K28" t="s">
+        <v>18</v>
+      </c>
+      <c r="M28" s="5">
+        <v>46297</v>
+      </c>
+      <c r="N28" t="s">
+        <v>26</v>
+      </c>
+      <c r="O28" t="s">
+        <v>19</v>
+      </c>
+      <c r="P28" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.25">
@@ -781,10 +832,76 @@
         <v>13</v>
       </c>
       <c r="E29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F29" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="H29" s="5">
+        <v>46297</v>
+      </c>
+      <c r="I29" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29" t="s">
+        <v>19</v>
+      </c>
+      <c r="K29" t="s">
+        <v>18</v>
+      </c>
+      <c r="M29" s="5">
+        <v>46297</v>
+      </c>
+      <c r="N29" t="s">
+        <v>27</v>
+      </c>
+      <c r="O29" t="s">
+        <v>19</v>
+      </c>
+      <c r="P29" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="C31" s="5">
+        <v>46297</v>
+      </c>
+      <c r="D31" t="s">
+        <v>2</v>
+      </c>
+      <c r="E31" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="C32" s="5">
+        <v>46297</v>
+      </c>
+      <c r="D32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E32" t="s">
+        <v>19</v>
+      </c>
+      <c r="F32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C33" s="5">
+        <v>46297</v>
+      </c>
+      <c r="D33" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated the forensic tracking xlsx
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Forensic File Tracking\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Desktop\2026 Y3 BIT\trimester2\Capstone\BHB-Capstone\Forensic File Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A1BDDFE-A367-400D-A7C2-186AA66F5413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E417058A-1011-4D75-8BF6-E47D0EA2BB8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2910" windowWidth="29040" windowHeight="15990" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="29">
   <si>
     <t>File</t>
   </si>
@@ -124,6 +124,9 @@
   </si>
   <si>
     <t>28sepServiceScan.xml</t>
+  </si>
+  <si>
+    <t>SOIT Scan</t>
   </si>
 </sst>
 </file>
@@ -643,8 +646,26 @@
       <c r="F6" t="s">
         <v>11</v>
       </c>
+      <c r="H6" s="5">
+        <v>46298</v>
+      </c>
       <c r="I6" t="s">
         <v>24</v>
+      </c>
+      <c r="J6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P6" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
updated logs, updated file tracking document, added wireshark findings section to research report
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Forensic File Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A1BDDFE-A367-400D-A7C2-186AA66F5413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C3C182-6EA2-4C48-8B0D-4B43496BEE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2910" windowWidth="29040" windowHeight="15990" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
+    <workbookView xWindow="38475" yWindow="3780" windowWidth="28335" windowHeight="12705" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="30">
   <si>
     <t>File</t>
   </si>
@@ -124,6 +124,14 @@
   </si>
   <si>
     <t>28sepServiceScan.xml</t>
+  </si>
+  <si>
+    <t>WIRESHARK
+w/HammerheadV1.py</t>
+  </si>
+  <si>
+    <t>NMAP
+w/SilentCartographerV1.py</t>
   </si>
 </sst>
 </file>
@@ -558,7 +566,7 @@
     <col min="10" max="10" width="19.85546875" customWidth="1"/>
     <col min="11" max="11" width="22.5703125" customWidth="1"/>
     <col min="12" max="12" width="22.5703125" style="2" customWidth="1"/>
-    <col min="13" max="13" width="22.5703125" customWidth="1"/>
+    <col min="13" max="13" width="24.85546875" customWidth="1"/>
     <col min="14" max="14" width="21.140625" customWidth="1"/>
     <col min="15" max="15" width="17.5703125" customWidth="1"/>
     <col min="16" max="16" width="18.42578125" customWidth="1"/>
@@ -701,12 +709,12 @@
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
-      <c r="H25" s="1" t="s">
-        <v>6</v>
+      <c r="H25" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="I25" s="1"/>
-      <c r="M25" s="1" t="s">
-        <v>7</v>
+      <c r="M25" s="4" t="s">
+        <v>29</v>
       </c>
       <c r="N25" s="1"/>
     </row>

</xml_diff>

<commit_message>
added my contributions to the tracking file.
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Forensic File Tracking\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Desktop\2026 Y3 BIT\trimester2\Capstone\BHB-Capstone\Forensic File Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C3C182-6EA2-4C48-8B0D-4B43496BEE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC4066A4-166E-49FA-BFF5-E51E9B4A298F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38475" yWindow="3780" windowWidth="28335" windowHeight="12705" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="32">
   <si>
     <t>File</t>
   </si>
@@ -132,6 +132,12 @@
   <si>
     <t>NMAP
 w/SilentCartographerV1.py</t>
+  </si>
+  <si>
+    <t>SOITNetworkscan.xml</t>
+  </si>
+  <si>
+    <t>Sam</t>
   </si>
 </sst>
 </file>
@@ -651,8 +657,29 @@
       <c r="F6" t="s">
         <v>11</v>
       </c>
+      <c r="H6" s="5">
+        <v>46298</v>
+      </c>
       <c r="I6" t="s">
         <v>24</v>
+      </c>
+      <c r="J6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M6" s="5">
+        <v>46300</v>
+      </c>
+      <c r="N6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P6" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added foremost report + updated tracking sheet
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/Forensic File Tracking/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d87909e21b199fc/Documents/BHB-Capstone/Forensic File Tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{EC4066A4-166E-49FA-BFF5-E51E9B4A298F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAD34B1A-3FCB-483C-A7E8-1815E37221BA}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{EC4066A4-166E-49FA-BFF5-E51E9B4A298F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D782FF62-4710-4608-9C51-0940894BA1EE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="41">
   <si>
     <t>File</t>
   </si>
@@ -159,6 +159,12 @@
   </si>
   <si>
     <t>7h 15m</t>
+  </si>
+  <si>
+    <t>THREE.dd</t>
+  </si>
+  <si>
+    <t>21.5h</t>
   </si>
 </sst>
 </file>
@@ -260,10 +266,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -584,27 +586,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58C512E3-CCD5-4663-8B80-5D68DC0D3979}">
   <dimension ref="B2:T33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="22.42578125" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" customWidth="1"/>
-    <col min="6" max="7" width="21.7109375" customWidth="1"/>
-    <col min="8" max="8" width="22.5703125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="22.85546875" customWidth="1"/>
-    <col min="10" max="10" width="17.140625" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" customWidth="1"/>
-    <col min="12" max="13" width="22.5703125" customWidth="1"/>
-    <col min="14" max="14" width="22.5703125" style="2" customWidth="1"/>
-    <col min="15" max="15" width="24.85546875" customWidth="1"/>
-    <col min="16" max="16" width="21.140625" customWidth="1"/>
-    <col min="17" max="17" width="17.5703125" customWidth="1"/>
-    <col min="18" max="19" width="18.42578125" customWidth="1"/>
-    <col min="20" max="20" width="8.7109375" style="2"/>
+    <col min="3" max="3" width="16.7265625" customWidth="1"/>
+    <col min="4" max="4" width="22.453125" customWidth="1"/>
+    <col min="5" max="5" width="17.7265625" customWidth="1"/>
+    <col min="6" max="7" width="21.7265625" customWidth="1"/>
+    <col min="8" max="8" width="22.54296875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="22.81640625" customWidth="1"/>
+    <col min="10" max="10" width="17.1796875" customWidth="1"/>
+    <col min="11" max="11" width="19.81640625" customWidth="1"/>
+    <col min="12" max="13" width="22.54296875" customWidth="1"/>
+    <col min="14" max="14" width="22.54296875" style="2" customWidth="1"/>
+    <col min="15" max="15" width="24.81640625" customWidth="1"/>
+    <col min="16" max="16" width="21.1796875" customWidth="1"/>
+    <col min="17" max="17" width="17.54296875" customWidth="1"/>
+    <col min="18" max="19" width="18.453125" customWidth="1"/>
+    <col min="20" max="20" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -614,12 +616,12 @@
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
     </row>
-    <row r="3" spans="2:19" s="2" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:19" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:19" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:19" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
@@ -636,7 +638,7 @@
       </c>
       <c r="P4" s="1"/>
     </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
@@ -683,7 +685,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C6" s="5">
         <v>46288</v>
       </c>
@@ -730,30 +732,31 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="C7" s="5">
+        <v>46310</v>
+      </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
       </c>
       <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L7" t="s">
         <v>11</v>
-      </c>
-      <c r="I7" s="5">
-        <v>46296</v>
-      </c>
-      <c r="J7" t="s">
-        <v>22</v>
-      </c>
-      <c r="K7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L7" t="s">
-        <v>18</v>
-      </c>
-      <c r="M7" t="s">
-        <v>38</v>
       </c>
       <c r="O7" s="5">
         <v>46304</v>
@@ -771,7 +774,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C8" s="5">
         <v>46287</v>
       </c>
@@ -787,22 +790,37 @@
       <c r="G8" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="I8" s="5">
+        <v>46296</v>
+      </c>
+      <c r="J8" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" t="s">
+        <v>18</v>
+      </c>
+      <c r="M8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.35">
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.35">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="24" spans="2:19" s="2" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:19" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B24" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:19" ht="45.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:19" ht="29.5" thickTop="1" x14ac:dyDescent="0.35">
       <c r="C25" s="4" t="s">
         <v>21</v>
       </c>
@@ -819,7 +837,7 @@
       </c>
       <c r="P25" s="1"/>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
@@ -860,7 +878,7 @@
       </c>
       <c r="S26" s="1"/>
     </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C27" s="5">
         <v>46288</v>
       </c>
@@ -898,7 +916,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C28" s="5">
         <v>46288</v>
       </c>
@@ -936,7 +954,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C29" s="5">
         <v>46288</v>
       </c>
@@ -974,7 +992,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C31" s="5">
         <v>46297</v>
       </c>
@@ -988,7 +1006,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C32" s="5">
         <v>46297</v>
       </c>
@@ -1002,7 +1020,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C33" s="5">
         <v>46297</v>
       </c>

</xml_diff>

<commit_message>
added time taken to complete for AI section in seconds)
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d87909e21b199fc/Documents/BHB-Capstone/Forensic File Tracking/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Desktop\2026 Y3 BIT\trimester2\Capstone\BHB-Capstone\Forensic File Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{EC4066A4-166E-49FA-BFF5-E51E9B4A298F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D782FF62-4710-4608-9C51-0940894BA1EE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACB0F40-A37E-49F2-89FF-33804CF2A9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="51">
   <si>
     <t>File</t>
   </si>
@@ -165,6 +165,36 @@
   </si>
   <si>
     <t>21.5h</t>
+  </si>
+  <si>
+    <t>2h</t>
+  </si>
+  <si>
+    <t>19s</t>
+  </si>
+  <si>
+    <t>37s</t>
+  </si>
+  <si>
+    <t>45s</t>
+  </si>
+  <si>
+    <t>157s</t>
+  </si>
+  <si>
+    <t>115s</t>
+  </si>
+  <si>
+    <t>137s</t>
+  </si>
+  <si>
+    <t>103s</t>
+  </si>
+  <si>
+    <t>81s</t>
+  </si>
+  <si>
+    <t>99s</t>
   </si>
 </sst>
 </file>
@@ -586,27 +616,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58C512E3-CCD5-4663-8B80-5D68DC0D3979}">
   <dimension ref="B2:T33"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="16.7265625" customWidth="1"/>
-    <col min="4" max="4" width="22.453125" customWidth="1"/>
-    <col min="5" max="5" width="17.7265625" customWidth="1"/>
-    <col min="6" max="7" width="21.7265625" customWidth="1"/>
-    <col min="8" max="8" width="22.54296875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="22.81640625" customWidth="1"/>
-    <col min="10" max="10" width="17.1796875" customWidth="1"/>
-    <col min="11" max="11" width="19.81640625" customWidth="1"/>
-    <col min="12" max="13" width="22.54296875" customWidth="1"/>
-    <col min="14" max="14" width="22.54296875" style="2" customWidth="1"/>
-    <col min="15" max="15" width="24.81640625" customWidth="1"/>
-    <col min="16" max="16" width="21.1796875" customWidth="1"/>
-    <col min="17" max="17" width="17.54296875" customWidth="1"/>
-    <col min="18" max="19" width="18.453125" customWidth="1"/>
-    <col min="20" max="20" width="8.7265625" style="2"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="6" max="7" width="21.7109375" customWidth="1"/>
+    <col min="8" max="8" width="22.5703125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="22.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.140625" customWidth="1"/>
+    <col min="11" max="11" width="19.85546875" customWidth="1"/>
+    <col min="12" max="13" width="22.5703125" customWidth="1"/>
+    <col min="14" max="14" width="22.5703125" style="2" customWidth="1"/>
+    <col min="15" max="15" width="24.85546875" customWidth="1"/>
+    <col min="16" max="16" width="21.140625" customWidth="1"/>
+    <col min="17" max="17" width="17.5703125" customWidth="1"/>
+    <col min="18" max="19" width="18.42578125" customWidth="1"/>
+    <col min="20" max="20" width="8.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -616,12 +646,12 @@
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
     </row>
-    <row r="3" spans="2:19" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:19" s="2" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:19" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:19" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
@@ -638,7 +668,7 @@
       </c>
       <c r="P4" s="1"/>
     </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
@@ -685,7 +715,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C6" s="5">
         <v>46288</v>
       </c>
@@ -732,7 +762,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C7" s="5">
         <v>46310</v>
       </c>
@@ -774,7 +804,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C8" s="5">
         <v>46287</v>
       </c>
@@ -805,22 +835,37 @@
       <c r="M8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="O8" s="5">
+        <v>46313</v>
+      </c>
+      <c r="P8" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>14</v>
+      </c>
+      <c r="R8" t="s">
+        <v>18</v>
+      </c>
+      <c r="S8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="24" spans="2:19" s="2" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="2:19" s="2" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:19" ht="29.5" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:19" ht="45.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C25" s="4" t="s">
         <v>21</v>
       </c>
@@ -837,7 +882,7 @@
       </c>
       <c r="P25" s="1"/>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
@@ -850,7 +895,9 @@
       <c r="F26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G26" s="1"/>
+      <c r="G26" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="I26" s="1" t="s">
         <v>15</v>
       </c>
@@ -863,7 +910,9 @@
       <c r="L26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="M26" s="1"/>
+      <c r="M26" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="O26" s="1" t="s">
         <v>15</v>
       </c>
@@ -876,9 +925,11 @@
       <c r="R26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="S26" s="1"/>
-    </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="S26" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C27" s="5">
         <v>46288</v>
       </c>
@@ -891,6 +942,9 @@
       <c r="F27" t="s">
         <v>18</v>
       </c>
+      <c r="G27" t="s">
+        <v>42</v>
+      </c>
       <c r="I27" s="5">
         <v>46297</v>
       </c>
@@ -903,6 +957,9 @@
       <c r="L27" t="s">
         <v>18</v>
       </c>
+      <c r="M27" t="s">
+        <v>45</v>
+      </c>
       <c r="O27" s="5">
         <v>46297</v>
       </c>
@@ -915,8 +972,11 @@
       <c r="R27" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="28" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="S27" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C28" s="5">
         <v>46288</v>
       </c>
@@ -929,6 +989,9 @@
       <c r="F28" t="s">
         <v>18</v>
       </c>
+      <c r="G28" t="s">
+        <v>43</v>
+      </c>
       <c r="I28" s="5">
         <v>46297</v>
       </c>
@@ -941,6 +1004,9 @@
       <c r="L28" t="s">
         <v>18</v>
       </c>
+      <c r="M28" t="s">
+        <v>46</v>
+      </c>
       <c r="O28" s="5">
         <v>46297</v>
       </c>
@@ -953,8 +1019,11 @@
       <c r="R28" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="29" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="S28" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C29" s="5">
         <v>46288</v>
       </c>
@@ -967,6 +1036,9 @@
       <c r="F29" t="s">
         <v>18</v>
       </c>
+      <c r="G29" t="s">
+        <v>44</v>
+      </c>
       <c r="I29" s="5">
         <v>46297</v>
       </c>
@@ -979,6 +1051,9 @@
       <c r="L29" t="s">
         <v>18</v>
       </c>
+      <c r="M29" t="s">
+        <v>47</v>
+      </c>
       <c r="O29" s="5">
         <v>46297</v>
       </c>
@@ -991,8 +1066,11 @@
       <c r="R29" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="S29" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C31" s="5">
         <v>46297</v>
       </c>
@@ -1006,7 +1084,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C32" s="5">
         <v>46297</v>
       </c>
@@ -1020,7 +1098,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="3:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C33" s="5">
         <v>46297</v>
       </c>

</xml_diff>

<commit_message>
Changed error in file tracking sheet
</commit_message>
<xml_diff>
--- a/Forensic File Tracking/Forensic File Tracking.xlsx
+++ b/Forensic File Tracking/Forensic File Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d87909e21b199fc/Documents/BHB-Capstone/Forensic File Tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{5ACB0F40-A37E-49F2-89FF-33804CF2A9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C034B6EE-3DA4-4760-BFDB-12718C6A7D5A}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{5ACB0F40-A37E-49F2-89FF-33804CF2A9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6AC6CA9-EF5A-4568-B076-BE0F0E9787B3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{3B890713-A654-4D72-B0E4-64232C3467A8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="51">
   <si>
     <t>File</t>
   </si>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t>AI MODEL</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>Olivia Hey</t>
@@ -673,7 +670,7 @@
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>0</v>
@@ -685,10 +682,10 @@
         <v>4</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>0</v>
@@ -700,10 +697,10 @@
         <v>4</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>0</v>
@@ -715,7 +712,7 @@
         <v>4</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.35">
@@ -729,40 +726,40 @@
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5">
         <v>46298</v>
       </c>
       <c r="J6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O6" s="5">
         <v>46300</v>
       </c>
       <c r="P6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.35">
@@ -770,44 +767,46 @@
         <v>46310</v>
       </c>
       <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
         <v>39</v>
       </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" s="5"/>
+      <c r="I7" s="5">
+        <v>46317</v>
+      </c>
       <c r="J7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L7" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="M7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O7" s="5">
         <v>46304</v>
       </c>
       <c r="P7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q7" t="s">
         <v>3</v>
       </c>
       <c r="R7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="2:19" x14ac:dyDescent="0.35">
@@ -815,46 +814,46 @@
         <v>46287</v>
       </c>
       <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
         <v>13</v>
       </c>
-      <c r="E8" t="s">
-        <v>14</v>
-      </c>
       <c r="F8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I8" s="5">
         <v>46296</v>
       </c>
       <c r="J8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K8" t="s">
         <v>3</v>
       </c>
       <c r="L8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O8" s="5">
         <v>46313</v>
       </c>
       <c r="P8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.35">
@@ -873,39 +872,39 @@
     </row>
     <row r="25" spans="2:19" ht="29.5" thickTop="1" x14ac:dyDescent="0.35">
       <c r="C25" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="I25" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J25" s="1"/>
       <c r="O25" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="P25" s="1"/>
     </row>
     <row r="26" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C26" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>0</v>
@@ -917,10 +916,10 @@
         <v>4</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P26" s="1" t="s">
         <v>0</v>
@@ -932,7 +931,7 @@
         <v>4</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="2:19" x14ac:dyDescent="0.35">
@@ -943,43 +942,43 @@
         <v>2</v>
       </c>
       <c r="E27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I27" s="5">
         <v>46297</v>
       </c>
       <c r="J27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="O27" s="5">
         <v>46297</v>
       </c>
       <c r="P27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="R27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="2:19" x14ac:dyDescent="0.35">
@@ -987,46 +986,46 @@
         <v>46288</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I28" s="5">
         <v>46297</v>
       </c>
       <c r="J28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="O28" s="5">
         <v>46297</v>
       </c>
       <c r="P28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="Q28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="R28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="2:19" x14ac:dyDescent="0.35">
@@ -1034,46 +1033,46 @@
         <v>46288</v>
       </c>
       <c r="D29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I29" s="5">
         <v>46297</v>
       </c>
       <c r="J29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M29" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="O29" s="5">
         <v>46297</v>
       </c>
       <c r="P29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Q29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="R29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S29" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="2:19" x14ac:dyDescent="0.35">
@@ -1084,10 +1083,10 @@
         <v>2</v>
       </c>
       <c r="E31" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="2:19" x14ac:dyDescent="0.35">
@@ -1095,13 +1094,13 @@
         <v>46297</v>
       </c>
       <c r="D32" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E32" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="3:6" x14ac:dyDescent="0.35">
@@ -1109,13 +1108,13 @@
         <v>46297</v>
       </c>
       <c r="D33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>